<commit_message>
Add Excel 05 Budget Tracking - Budget vs Actual Variance Analysis
</commit_message>
<xml_diff>
--- a/excel/04_supplier_evaluation/04_supplier_evaluation.xlsx
+++ b/excel/04_supplier_evaluation/04_supplier_evaluation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c832e410b044d57/Documents/data_analysis_projects/excel/04_supplier_evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="336" documentId="11_C24A40B9DC05913DA6F65445B1759392D2C57E61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E978EFD-75BC-433A-BDEF-16030861089B}"/>
+  <xr:revisionPtr revIDLastSave="340" documentId="11_C24A40B9DC05913DA6F65445B1759392D2C57E61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8B6B093-EC55-460F-964C-210A71D234CE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>quality</t>
   </si>
@@ -244,15 +244,18 @@
   <si>
     <t>TOP TIER SUPPLIERS</t>
   </si>
+  <si>
+    <t>Data source: Dynamic Inventory Analytics · Kaggle · Kaizen Analytics · kaggle.com/datasets/andrewniko/dynamic-inventory-dataset-kaizen-analytics</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="175" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,6 +324,13 @@
     <font>
       <i/>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -405,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -428,13 +438,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -443,22 +468,10 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -466,6 +479,16 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="6" tint="0.39994506668294322"/>
@@ -483,16 +506,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -514,6 +527,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4475,11 +4492,11 @@
         <v>0.70421138211382117</v>
       </c>
       <c r="C2">
-        <f>RANK(B2,$B$2:$B$36,0)</f>
+        <f t="shared" ref="C2:C36" si="0">RANK(B2,$B$2:$B$36,0)</f>
         <v>1</v>
       </c>
       <c r="D2" t="str">
-        <f>IF(C2&lt;=7,"Preferred",IF(C2&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" ref="D2:D36" si="1">IF(C2&lt;=7,"Preferred",IF(C2&lt;=21,"Approved","Conditional"))</f>
         <v>Preferred</v>
       </c>
       <c r="E2">
@@ -4509,11 +4526,11 @@
         <v>0.68053658536585371</v>
       </c>
       <c r="C3">
-        <f>RANK(B3,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="D3" t="str">
-        <f>IF(C3&lt;=7,"Preferred",IF(C3&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Preferred</v>
       </c>
       <c r="E3">
@@ -4543,11 +4560,11 @@
         <v>0.65834146341463418</v>
       </c>
       <c r="C4">
-        <f>RANK(B4,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="D4" t="str">
-        <f>IF(C4&lt;=7,"Preferred",IF(C4&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Preferred</v>
       </c>
       <c r="E4">
@@ -4577,11 +4594,11 @@
         <v>0.62347967479674804</v>
       </c>
       <c r="C5">
-        <f>RANK(B5,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="D5" t="str">
-        <f>IF(C5&lt;=7,"Preferred",IF(C5&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Preferred</v>
       </c>
       <c r="E5">
@@ -4611,11 +4628,11 @@
         <v>0.61860162601626023</v>
       </c>
       <c r="C6">
-        <f>RANK(B6,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="D6" t="str">
-        <f>IF(C6&lt;=7,"Preferred",IF(C6&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Preferred</v>
       </c>
       <c r="E6">
@@ -4645,11 +4662,11 @@
         <v>0.6014959349593495</v>
       </c>
       <c r="C7">
-        <f>RANK(B7,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="D7" t="str">
-        <f>IF(C7&lt;=7,"Preferred",IF(C7&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Preferred</v>
       </c>
       <c r="E7">
@@ -4679,11 +4696,11 @@
         <v>0.59533333333333327</v>
       </c>
       <c r="C8">
-        <f>RANK(B8,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="D8" t="str">
-        <f>IF(C8&lt;=7,"Preferred",IF(C8&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Preferred</v>
       </c>
       <c r="E8">
@@ -4713,11 +4730,11 @@
         <v>0.57853658536585373</v>
       </c>
       <c r="C9">
-        <f>RANK(B9,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D9" t="str">
-        <f>IF(C9&lt;=7,"Preferred",IF(C9&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E9">
@@ -4747,11 +4764,11 @@
         <v>0.57284552845528458</v>
       </c>
       <c r="C10">
-        <f>RANK(B10,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="D10" t="str">
-        <f>IF(C10&lt;=7,"Preferred",IF(C10&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E10">
@@ -4781,11 +4798,11 @@
         <v>0.5547804878048781</v>
       </c>
       <c r="C11">
-        <f>RANK(B11,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D11" t="str">
-        <f>IF(C11&lt;=7,"Preferred",IF(C11&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E11">
@@ -4815,11 +4832,11 @@
         <v>0.53559349593495942</v>
       </c>
       <c r="C12">
-        <f>RANK(B12,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="D12" t="str">
-        <f>IF(C12&lt;=7,"Preferred",IF(C12&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E12">
@@ -4849,11 +4866,11 @@
         <v>0.53435772357723588</v>
       </c>
       <c r="C13">
-        <f>RANK(B13,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="D13" t="str">
-        <f>IF(C13&lt;=7,"Preferred",IF(C13&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E13">
@@ -4883,11 +4900,11 @@
         <v>0.52541463414634149</v>
       </c>
       <c r="C14">
-        <f>RANK(B14,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="D14" t="str">
-        <f>IF(C14&lt;=7,"Preferred",IF(C14&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E14">
@@ -4917,11 +4934,11 @@
         <v>0.52295934959349599</v>
       </c>
       <c r="C15">
-        <f>RANK(B15,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="D15" t="str">
-        <f>IF(C15&lt;=7,"Preferred",IF(C15&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E15">
@@ -4951,11 +4968,11 @@
         <v>0.52284552845528465</v>
       </c>
       <c r="C16">
-        <f>RANK(B16,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="D16" t="str">
-        <f>IF(C16&lt;=7,"Preferred",IF(C16&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E16">
@@ -4985,11 +5002,11 @@
         <v>0.5102439024390244</v>
       </c>
       <c r="C17">
-        <f>RANK(B17,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="D17" t="str">
-        <f>IF(C17&lt;=7,"Preferred",IF(C17&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E17">
@@ -5019,11 +5036,11 @@
         <v>0.49260162601626017</v>
       </c>
       <c r="C18">
-        <f>RANK(B18,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="D18" t="str">
-        <f>IF(C18&lt;=7,"Preferred",IF(C18&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E18">
@@ -5053,11 +5070,11 @@
         <v>0.48671544715447157</v>
       </c>
       <c r="C19">
-        <f>RANK(B19,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="D19" t="str">
-        <f>IF(C19&lt;=7,"Preferred",IF(C19&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E19">
@@ -5087,11 +5104,11 @@
         <v>0.46421138211382112</v>
       </c>
       <c r="C20">
-        <f>RANK(B20,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="D20" t="str">
-        <f>IF(C20&lt;=7,"Preferred",IF(C20&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E20">
@@ -5121,11 +5138,11 @@
         <v>0.43196747967479676</v>
       </c>
       <c r="C21">
-        <f>RANK(B21,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="D21" t="str">
-        <f>IF(C21&lt;=7,"Preferred",IF(C21&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E21">
@@ -5155,11 +5172,11 @@
         <v>0.43196747967479676</v>
       </c>
       <c r="C22">
-        <f>RANK(B22,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="D22" t="str">
-        <f>IF(C22&lt;=7,"Preferred",IF(C22&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Approved</v>
       </c>
       <c r="E22">
@@ -5189,11 +5206,11 @@
         <v>0.43126829268292682</v>
       </c>
       <c r="C23">
-        <f>RANK(B23,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="D23" t="str">
-        <f>IF(C23&lt;=7,"Preferred",IF(C23&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E23">
@@ -5223,11 +5240,11 @@
         <v>0.423869918699187</v>
       </c>
       <c r="C24">
-        <f>RANK(B24,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="D24" t="str">
-        <f>IF(C24&lt;=7,"Preferred",IF(C24&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E24">
@@ -5257,11 +5274,11 @@
         <v>0.39921951219512197</v>
       </c>
       <c r="C25">
-        <f>RANK(B25,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="D25" t="str">
-        <f>IF(C25&lt;=7,"Preferred",IF(C25&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E25">
@@ -5291,11 +5308,11 @@
         <v>0.38871544715447159</v>
       </c>
       <c r="C26">
-        <f>RANK(B26,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="D26" t="str">
-        <f>IF(C26&lt;=7,"Preferred",IF(C26&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E26">
@@ -5325,11 +5342,11 @@
         <v>0.37029268292682926</v>
       </c>
       <c r="C27">
-        <f>RANK(B27,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="D27" t="str">
-        <f>IF(C27&lt;=7,"Preferred",IF(C27&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E27">
@@ -5359,11 +5376,11 @@
         <v>0.36559349593495938</v>
       </c>
       <c r="C28">
-        <f>RANK(B28,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="D28" t="str">
-        <f>IF(C28&lt;=7,"Preferred",IF(C28&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E28">
@@ -5393,11 +5410,11 @@
         <v>0.35666666666666669</v>
       </c>
       <c r="C29">
-        <f>RANK(B29,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="D29" t="str">
-        <f>IF(C29&lt;=7,"Preferred",IF(C29&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E29">
@@ -5427,11 +5444,11 @@
         <v>0.34756097560975613</v>
       </c>
       <c r="C30">
-        <f>RANK(B30,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="D30" t="str">
-        <f>IF(C30&lt;=7,"Preferred",IF(C30&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E30">
@@ -5461,11 +5478,11 @@
         <v>0.34373983739837394</v>
       </c>
       <c r="C31">
-        <f>RANK(B31,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="D31" t="str">
-        <f>IF(C31&lt;=7,"Preferred",IF(C31&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E31">
@@ -5495,11 +5512,11 @@
         <v>0.3256910569105691</v>
       </c>
       <c r="C32">
-        <f>RANK(B32,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="D32" t="str">
-        <f>IF(C32&lt;=7,"Preferred",IF(C32&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E32">
@@ -5529,11 +5546,11 @@
         <v>0.30734959349593494</v>
       </c>
       <c r="C33">
-        <f>RANK(B33,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="D33" t="str">
-        <f>IF(C33&lt;=7,"Preferred",IF(C33&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E33">
@@ -5563,11 +5580,11 @@
         <v>0.29533333333333334</v>
       </c>
       <c r="C34">
-        <f>RANK(B34,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="D34" t="str">
-        <f>IF(C34&lt;=7,"Preferred",IF(C34&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E34">
@@ -5597,11 +5614,11 @@
         <v>0.2797073170731707</v>
       </c>
       <c r="C35">
-        <f>RANK(B35,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="D35" t="str">
-        <f>IF(C35&lt;=7,"Preferred",IF(C35&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E35">
@@ -5631,11 +5648,11 @@
         <v>0.24980487804878054</v>
       </c>
       <c r="C36">
-        <f>RANK(B36,$B$2:$B$36,0)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="D36" t="str">
-        <f>IF(C36&lt;=7,"Preferred",IF(C36&lt;=21,"Approved","Conditional"))</f>
+        <f t="shared" si="1"/>
         <v>Conditional</v>
       </c>
       <c r="E36">
@@ -5667,7 +5684,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA9BF2E0-4631-4C31-8339-005972E52085}">
-  <dimension ref="B2:M33"/>
+  <dimension ref="B2:M35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.21875" customWidth="1"/>
@@ -5676,748 +5693,740 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="21" x14ac:dyDescent="0.4">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
     </row>
     <row r="3" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10" t="s">
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10" t="s">
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10" t="s">
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B6" s="11">
+      <c r="B6" s="18">
         <f>COUNTA(Scoring!$A$2:$A$36)</f>
         <v>35</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11">
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18">
         <f>COUNTIF(Scoring!$D$2:$D$36,"Preferred")</f>
         <v>7</v>
       </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11">
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18">
         <f>COUNTIF(Scoring!$D$2:$D$36,"Approved")</f>
         <v>14</v>
       </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11">
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18">
         <f>COUNTIF(Scoring!$D$2:$D$36,"Conditional")</f>
         <v>14</v>
       </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12" t="s">
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12" t="s">
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12" t="s">
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
     </row>
     <row r="10" spans="2:13" ht="21" x14ac:dyDescent="0.4">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10" t="s">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10" t="s">
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B12" s="14" t="str">
+      <c r="B12" s="11" t="str">
         <f>Weights!A2</f>
         <v>quality</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="18">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.45714285714285713</v>
       </c>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="14" t="str">
-        <f ca="1">IF(G12&gt;=0.7,"Strong",IF(G12&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="11" t="str">
+        <f t="shared" ref="J12:J23" ca="1" si="0">IF(G12&gt;=0.7,"Strong",IF(G12&gt;=0.4,"Moderate","Weak"))</f>
         <v>Moderate</v>
       </c>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B13" s="14" t="str">
+      <c r="B13" s="11" t="str">
         <f>Weights!A3</f>
         <v>quantity</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="18">
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.31199999999999994</v>
       </c>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="14" t="str">
-        <f ca="1">IF(G13&gt;=0.7,"Strong",IF(G13&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Weak</v>
       </c>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="14"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B14" s="14" t="str">
+      <c r="B14" s="11" t="str">
         <f>Weights!A4</f>
         <v>conditions and method of payment</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="18">
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.47857142857142859</v>
       </c>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="14" t="str">
-        <f ca="1">IF(G14&gt;=0.7,"Strong",IF(G14&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B15" s="14" t="str">
+      <c r="B15" s="11" t="str">
         <f>Weights!A5</f>
         <v>serviceability and communicativeness</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="18">
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.4904761904761904</v>
       </c>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="14" t="str">
-        <f ca="1">IF(G15&gt;=0.7,"Strong",IF(G15&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B16" s="14" t="str">
+      <c r="B16" s="11" t="str">
         <f>Weights!A6</f>
         <v>reputation and competence</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="18">
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.43428571428571422</v>
       </c>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="14" t="str">
-        <f ca="1">IF(G16&gt;=0.7,"Strong",IF(G16&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B17" s="14" t="str">
+      <c r="B17" s="11" t="str">
         <f>Weights!A7</f>
         <v>flexibility</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="18">
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.46666666666666662</v>
       </c>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="14" t="str">
-        <f ca="1">IF(G17&gt;=0.7,"Strong",IF(G17&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B18" s="14" t="str">
+      <c r="B18" s="11" t="str">
         <f>Weights!A8</f>
         <v>financial condition</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="18">
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.47142857142857142</v>
       </c>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="14" t="str">
-        <f ca="1">IF(G18&gt;=0.7,"Strong",IF(G18&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B19" s="14" t="str">
+      <c r="B19" s="11" t="str">
         <f>Weights!A9</f>
         <v>condition of assets</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="18">
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.54285714285714282</v>
       </c>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="14" t="str">
-        <f ca="1">IF(G19&gt;=0.7,"Strong",IF(G19&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="14"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B20" s="14" t="str">
+      <c r="B20" s="11" t="str">
         <f>Weights!A10</f>
         <v>business results and employees</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="18">
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.43999999999999995</v>
       </c>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="14" t="str">
-        <f ca="1">IF(G20&gt;=0.7,"Strong",IF(G20&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B21" s="14" t="str">
+      <c r="B21" s="11" t="str">
         <f>Weights!A11</f>
         <v>price</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="18">
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.53714285714285726</v>
       </c>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="14" t="str">
-        <f ca="1">IF(G21&gt;=0.7,"Strong",IF(G21&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B22" s="14" t="str">
+      <c r="B22" s="11" t="str">
         <f>Weights!A12</f>
         <v>delivery time</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="18">
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.45714285714285713</v>
       </c>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="14" t="str">
-        <f ca="1">IF(G22&gt;=0.7,"Strong",IF(G22&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Moderate</v>
       </c>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="11"/>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B23" s="14" t="str">
+      <c r="B23" s="11" t="str">
         <f>Weights!A13</f>
         <v>location and traffic</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="18">
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="12">
         <f ca="1">AVERAGE(OFFSET('Normalized Data'!$B$2:$B$36,0,ROW()-12))</f>
         <v>0.75958188153310113</v>
       </c>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="14" t="str">
-        <f ca="1">IF(G23&gt;=0.7,"Strong",IF(G23&gt;=0.4,"Moderate","Weak"))</f>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="11" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>Strong</v>
       </c>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-      <c r="M23" s="14"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
     </row>
     <row r="25" spans="2:13" ht="21" x14ac:dyDescent="0.4">
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B26" s="10" t="str">
+      <c r="B26" s="13" t="str">
         <f>Scoring!A1</f>
         <v>Supplier ID</v>
       </c>
-      <c r="C26" s="10"/>
-      <c r="D26" s="13" t="s">
+      <c r="C26" s="13"/>
+      <c r="D26" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="13" t="s">
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10" t="s">
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="M26" s="10"/>
+      <c r="M26" s="13"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B27" s="17">
+      <c r="B27" s="14">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(1,Scoring!$C$2:$C$36,0))</f>
         <v>9</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="16">
+      <c r="C27" s="14"/>
+      <c r="D27" s="10">
         <f>VLOOKUP(B27, Scoring!A2:B36, 2, FALSE)</f>
         <v>0.70421138211382117</v>
       </c>
-      <c r="E27" s="14" t="str">
+      <c r="E27" s="11" t="str">
         <f>VLOOKUP(B27, Scoring!A2:H36, 7, FALSE)</f>
         <v>quality</v>
       </c>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="15">
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="9">
         <f>VLOOKUP(B27, Scoring!A2:H36, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I27" s="14" t="str">
+      <c r="I27" s="11" t="str">
         <f>VLOOKUP(B27, Scoring!A2:H36, 8, FALSE)</f>
         <v>business results and employees</v>
       </c>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="18">
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="12">
         <f>VLOOKUP(B27, Scoring!A2:H36, 6, FALSE)</f>
         <v>0.2</v>
       </c>
-      <c r="M27" s="18"/>
+      <c r="M27" s="12"/>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B28" s="19">
+      <c r="B28" s="15">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(2,Scoring!$C$2:$C$36,0))</f>
         <v>24</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="16">
+      <c r="C28" s="16"/>
+      <c r="D28" s="10">
         <f>VLOOKUP(B28, Scoring!A3:B37, 2, FALSE)</f>
         <v>0.68053658536585371</v>
       </c>
-      <c r="E28" s="14" t="str">
+      <c r="E28" s="11" t="str">
         <f>VLOOKUP(B28, Scoring!A3:H37, 7, FALSE)</f>
         <v>reputation and competence</v>
       </c>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="15">
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="9">
         <f>VLOOKUP(B28, Scoring!A3:H37, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I28" s="14" t="str">
+      <c r="I28" s="11" t="str">
         <f>VLOOKUP(B28, Scoring!A3:H37, 8, FALSE)</f>
         <v>quantity</v>
       </c>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="18">
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="12">
         <f>VLOOKUP(B28, Scoring!A3:H37, 6, FALSE)</f>
         <v>0.30666666666666664</v>
       </c>
-      <c r="M28" s="18"/>
+      <c r="M28" s="12"/>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B29" s="19">
+      <c r="B29" s="15">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(3,Scoring!$C$2:$C$36,0))</f>
         <v>14</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="16">
+      <c r="C29" s="16"/>
+      <c r="D29" s="10">
         <f>VLOOKUP(B29, Scoring!A4:B38, 2, FALSE)</f>
         <v>0.65834146341463418</v>
       </c>
-      <c r="E29" s="14" t="str">
+      <c r="E29" s="11" t="str">
         <f>VLOOKUP(B29, Scoring!A4:H38, 7, FALSE)</f>
         <v>conditions and method of payment</v>
       </c>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="15">
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="9">
         <f>VLOOKUP(B29, Scoring!A4:H38, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I29" s="14" t="str">
+      <c r="I29" s="11" t="str">
         <f>VLOOKUP(B29, Scoring!A4:H38, 8, FALSE)</f>
         <v>quantity</v>
       </c>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="18">
+      <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
+      <c r="L29" s="12">
         <f>VLOOKUP(B29, Scoring!A4:H38, 6, FALSE)</f>
         <v>0.44</v>
       </c>
-      <c r="M29" s="18"/>
+      <c r="M29" s="12"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B30" s="19">
+      <c r="B30" s="15">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(4,Scoring!$C$2:$C$36,0))</f>
         <v>27</v>
       </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="16">
+      <c r="C30" s="16"/>
+      <c r="D30" s="10">
         <f>VLOOKUP(B30, Scoring!A5:B39, 2, FALSE)</f>
         <v>0.62347967479674804</v>
       </c>
-      <c r="E30" s="14" t="str">
+      <c r="E30" s="11" t="str">
         <f>VLOOKUP(B30, Scoring!A5:H39, 7, FALSE)</f>
         <v>serviceability and communicativeness</v>
       </c>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="15">
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="9">
         <f>VLOOKUP(B30, Scoring!A5:H39, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I30" s="14" t="str">
+      <c r="I30" s="11" t="str">
         <f>VLOOKUP(B30, Scoring!A5:H39, 8, FALSE)</f>
         <v>quality</v>
       </c>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="18">
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="12">
         <f>VLOOKUP(B30, Scoring!A5:H39, 6, FALSE)</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="M30" s="18"/>
+      <c r="M30" s="12"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B31" s="19">
+      <c r="B31" s="15">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(5,Scoring!$C$2:$C$36,0))</f>
         <v>25</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="16">
+      <c r="C31" s="16"/>
+      <c r="D31" s="10">
         <f>VLOOKUP(B31, Scoring!A6:B40, 2, FALSE)</f>
         <v>0.61860162601626023</v>
       </c>
-      <c r="E31" s="14" t="str">
+      <c r="E31" s="11" t="str">
         <f>VLOOKUP(B31, Scoring!A6:H40, 7, FALSE)</f>
         <v>reputation and competence</v>
       </c>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="15">
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="9">
         <f>VLOOKUP(B31, Scoring!A6:H40, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I31" s="14" t="str">
+      <c r="I31" s="11" t="str">
         <f>VLOOKUP(B31, Scoring!A6:H40, 8, FALSE)</f>
         <v>quality</v>
       </c>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="18">
+      <c r="J31" s="11"/>
+      <c r="K31" s="11"/>
+      <c r="L31" s="12">
         <f>VLOOKUP(B31, Scoring!A6:H40, 6, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="M31" s="18"/>
+      <c r="M31" s="12"/>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B32" s="19">
+      <c r="B32" s="15">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(6,Scoring!$C$2:$C$36,0))</f>
         <v>13</v>
       </c>
-      <c r="C32" s="20"/>
-      <c r="D32" s="16">
+      <c r="C32" s="16"/>
+      <c r="D32" s="10">
         <f>VLOOKUP(B32, Scoring!A7:B41, 2, FALSE)</f>
         <v>0.6014959349593495</v>
       </c>
-      <c r="E32" s="14" t="str">
+      <c r="E32" s="11" t="str">
         <f>VLOOKUP(B32, Scoring!A7:H41, 7, FALSE)</f>
         <v>conditions and method of payment</v>
       </c>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="15">
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="9">
         <f>VLOOKUP(B32, Scoring!A7:H41, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I32" s="14" t="str">
+      <c r="I32" s="11" t="str">
         <f>VLOOKUP(B32, Scoring!A7:H41, 8, FALSE)</f>
         <v>quantity</v>
       </c>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="18">
+      <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
+      <c r="L32" s="12">
         <f>VLOOKUP(B32, Scoring!A7:H41, 6, FALSE)</f>
         <v>9.3333333333333338E-2</v>
       </c>
-      <c r="M32" s="18"/>
+      <c r="M32" s="12"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B33" s="19">
+      <c r="B33" s="15">
         <f>INDEX(Scoring!$A$2:$A$36,MATCH(7,Scoring!$C$2:$C$36,0))</f>
         <v>16</v>
       </c>
-      <c r="C33" s="20"/>
-      <c r="D33" s="16">
+      <c r="C33" s="16"/>
+      <c r="D33" s="10">
         <f>VLOOKUP(B33, Scoring!A8:B42, 2, FALSE)</f>
         <v>0.59533333333333327</v>
       </c>
-      <c r="E33" s="14" t="str">
+      <c r="E33" s="11" t="str">
         <f>VLOOKUP(B33, Scoring!A8:H42, 7, FALSE)</f>
         <v>quality</v>
       </c>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="15">
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="9">
         <f>VLOOKUP(B33, Scoring!A8:H42, 5, FALSE)</f>
         <v>1</v>
       </c>
-      <c r="I33" s="14" t="str">
+      <c r="I33" s="11" t="str">
         <f>VLOOKUP(B33, Scoring!A8:H42, 8, FALSE)</f>
         <v>location and traffic</v>
       </c>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="18">
+      <c r="J33" s="11"/>
+      <c r="K33" s="11"/>
+      <c r="L33" s="12">
         <f>VLOOKUP(B33, Scoring!A8:H42, 6, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="M33" s="18"/>
+      <c r="M33" s="12"/>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B35" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+      <c r="M35" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="87">
-    <mergeCell ref="J18:M18"/>
-    <mergeCell ref="J19:M19"/>
-    <mergeCell ref="J20:M20"/>
-    <mergeCell ref="J21:M21"/>
-    <mergeCell ref="J22:M22"/>
-    <mergeCell ref="J23:M23"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="J12:M12"/>
-    <mergeCell ref="J13:M13"/>
-    <mergeCell ref="J14:M14"/>
-    <mergeCell ref="J15:M15"/>
-    <mergeCell ref="J16:M16"/>
-    <mergeCell ref="J17:M17"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:M11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
+  <mergeCells count="88">
+    <mergeCell ref="B35:M35"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="B10:M10"/>
+    <mergeCell ref="B6:D7"/>
+    <mergeCell ref="E6:G7"/>
+    <mergeCell ref="H6:J7"/>
+    <mergeCell ref="K6:M7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="I32:K32"/>
     <mergeCell ref="I33:K33"/>
@@ -6434,43 +6443,66 @@
     <mergeCell ref="E26:G26"/>
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="E33:G33"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="E32:G32"/>
     <mergeCell ref="B25:M25"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="B10:M10"/>
-    <mergeCell ref="B6:D7"/>
-    <mergeCell ref="E6:G7"/>
-    <mergeCell ref="H6:J7"/>
-    <mergeCell ref="K6:M7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:M3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J12:M12"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="J15:M15"/>
+    <mergeCell ref="J16:M16"/>
+    <mergeCell ref="J23:M23"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="J18:M18"/>
+    <mergeCell ref="J19:M19"/>
+    <mergeCell ref="J20:M20"/>
+    <mergeCell ref="J21:M21"/>
+    <mergeCell ref="J22:M22"/>
   </mergeCells>
   <conditionalFormatting sqref="J12:J23">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"Strong"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J12:J23">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Weak"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Moderate"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"Strong"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>